<commit_message>
Update to include data across multiple experiments
</commit_message>
<xml_diff>
--- a/Cell survival results/Analysis Results 16 October/Proton high.xlsx
+++ b/Cell survival results/Analysis Results 16 October/Proton high.xlsx
@@ -446,17 +446,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Count 1</t>
+          <t>Count_1</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Count 2</t>
+          <t>Count_2</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Count 3</t>
+          <t>Count_3</t>
         </is>
       </c>
     </row>

</xml_diff>